<commit_message>
feat(F-NAR-019): ATOM-DIF.BES.001-01 Les cartes de Sarah
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.001-01.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.001-01.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>La tortue de Sarah</t>
+          <t>Les cartes de Sarah</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>classe, tapis, puis maison</t>
+          <t>école, manteaux en rang, bottes, vitre floue, doigt qui dessine, cartes sur le tapis</t>
         </is>
       </c>
     </row>
@@ -688,7 +688,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sarah, Raphaël, papa, maman</t>
+          <t>Sarah, papa, maman</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah veut faire marcher la carte tortue jusqu'au soleil de la vitre. Raphaël reste près du mur. Elle répète. Il observe d'abord. La tortue arrive.</t>
+          <t>La vitre de la classe est floue. Un doigt y a tracé un soleil. Sur une carte, un éclat de carte brille. Sarah veut parler aux cartes maintenant. Sa voix part trop fort : les cartes glissent. Elle refuse de foncer, observe, dit le mot plus bas. On le dit comme elle. Merci vécu. Un éclat de carte reste pâle.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Un soleil de doigt dort sur la vitre. Il a trois rayons, un peu flous. Le tapis sent encore le savon. Une carte dépasse d'un sac. C'est une oreille de chat, toute grise. Tu as vu le soleil, Sarah ? Il est sur la vitre. Il a trois rayons. Oui. Un petit soleil de doigt. En ce moment, papa ouvre la porte. Sarah entre avec lui. Les chaussures font un bruit doux. Je veux la tortue. Elle va jusqu'au soleil. Tu la fais marcher, alors. Des cartes d'animaux attendent sur le tapis. Un sac est ouvert, tout bas. Raphaël reste près du mur. Ses mains touchent le crépi, tout doux. Il ne vient pas encore. Raphaël. Tu viens ? Raphaël ne bouge pas. Il regarde le sac, sans avancer. Il a besoin de calme. Tu peux dire comment on joue. Sarah s'arrête au bord du tapis. La carte du chat dépasse encore. Le soleil de doigt attend sur la vitre.</t>
+          <t>La vitre de la classe est floue. Un doigt y a tracé un soleil rond. Il a trois rayons, papa. Tu le vois, Sarah ? Les manteaux pendent en rang, près du mur. La laine sent un peu la pluie. Ton manteau va là, dans le rang. Les bottes font une petite file. Les miennes sont rouges. Oui, les rouges, près de la porte. Tu tiens ma manche, Sarah ? Oui, papa. Un banc de bois attend sous les manteaux. Le bois est froid. C'est le banc de l'entrée. Le tapis de la classe attend, un peu rêche. Des cartes d'animaux y sont posées, faces ouvertes. Des bêtes, maman ! Tu les vois, sur le tapis ? Une carte montre un chat, les oreilles hautes. Le chat, je le vois. À côté, une tortue garde la tête rentrée. Sur la carte, un éclat de carte brille. Il brille, papa. Tu le vois, sur le papier ? Sarah touche l'éclat de carte. Le papier est lisse, un peu froid. Elle est froide, la tortue. Je lui parle, maintenant ! Tu restes près de nous ? Oui, maman. Tu lui parles, à la tortue ? Oui, très fort ! En ce moment, Sarah se penche sur les cartes. Tortue, tu marches ! Sa voix part trop fort, trop vite. Les cartes glissent sur le tapis. Oh. La tortue disparaît sous une autre carte. L'éclat n'est plus là. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je la prends ! La carte est sous les autres. Tu la vois, Sarah ? Les épaules de Sarah tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Un soleil de doigt dort sur la vitre. Il a trois rayons, un peu flous. Le tapis sent encore le savon. Une carte dépasse d'un sac. C'est une oreille de chat, toute grise. Tu as vu le soleil, Sarah ? Il est sur la vitre. Il a trois rayons. Oui. Un petit soleil de doigt. En ce moment, papa ouvre la porte. Sarah entre avec lui. Les chaussures font un bruit doux. Je veux la tortue. Elle va jusqu'au soleil. Tu la fais marcher, alors. Des cartes d'animaux attendent sur le tapis. Un sac est ouvert, tout bas. Raphaël reste près du mur. Ses mains touchent le crépi, tout doux. Il ne vient pas encore. Raphaël. Tu viens ? Raphaël ne bouge pas. Il regarde le sac, sans avancer. Il a besoin de calme. Tu peux dire comment on joue. Sarah s'arrête au bord du tapis. La carte du chat dépasse encore. Le soleil de doigt attend sur la vitre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La vitre de la classe est floue. Un doigt y a tracé un soleil rond. Il a trois rayons, papa. Tu le vois, Sarah ? Les manteaux pendent en rang, près du mur. La laine sent un peu la pluie. Ton manteau va là, dans le rang. Les bottes font une petite file. Les miennes sont rouges. Oui, les rouges, près de la porte. Tu tiens ma manche, Sarah ? Oui, papa. Un banc de bois attend sous les manteaux. Le bois est froid. C'est le banc de l'entrée. Le tapis de la classe attend, un peu rêche. Des cartes d'animaux y sont posées, faces ouvertes. Des bêtes, maman ! Tu les vois, sur le tapis ? Une carte montre un chat, les oreilles hautes. Le chat, je le vois. À côté, une tortue garde la tête rentrée. Sur la carte, un &lt;emphasis level="moderate"&gt;éclat de carte&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, sur le papier ? Sarah touche l'éclat de carte. Le papier est lisse, un peu froid. Elle est froide, la tortue. Je lui parle, maintenant ! Tu restes près de nous ? Oui, maman. Tu lui parles, à la tortue ? Oui, très fort ! En ce moment, Sarah se penche sur les cartes. Tortue, tu marches ! Sa voix part trop fort, trop vite. Les cartes glissent sur le tapis. Oh. La tortue disparaît sous une autre carte. L'éclat n'est plus là. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je la prends ! La carte est sous les autres. Tu la vois, Sarah ? Les épaules de Sarah tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Papa accompagne Zoé en classe. Sur le tapis, il y a un nouveau jeu. Des cartes d'animaux. Des petits sacs. La maîtresse explique. On pioche une carte. On imite l'animal, tout doux. Iris reste près du mur. Elle a besoin de plus de temps. Elle a besoin de calme. Zoé l'appelle. Iris ne vient pas. Papa est encore à la porte. Il dit : on peut &lt;emphasis&gt;répéter&lt;/emphasis&gt; la règle. On peut observer d'abord. Zoé va vers Iris. Elle parle doucement. Zoé dit : on pioche une carte. On imite l'animal. Puis on repose la carte. C'est répéter la règle. Iris écoute. Elle reste près du mur. Elle va observer d'abord. Zoé retourne au tapis. Elle pioche un chat. Elle marche sur la pointe des pieds. Iris regarde. Elle ne joue pas encore. C'est possible. La maîtresse dit : Iris peut observer d'abord. Le groupe continue. Un enfant pioche un oiseau. Il ouvre les bras, lentement. Iris sourit un peu. Zoé vient encore. Elle va répéter, une fois. Zoé dit : une carte, un animal, tout doux. Iris hoche la tête. Elle s'assoit au bord du tapis. Elle observe d'abord. Plus tard, elle tend la main. Elle pioche une carte. C'est une tortue. Iris avance très lentement. Zoé laisse l'espace. Papa, au fond, fait un petit signe. À la fin, Iris n'a fait qu'une carte. C'est assez. Zoé range les sacs. Papa dit : tu as su répéter. Iris a pu observer d'abord. Le calme a aidé. [pause]</t>
+          <t>La vitre de la classe est floue. Un doigt y a tracé un soleil rond. Il a trois rayons, papa. Tu le vois, Sarah ? Les manteaux pendent en rang, près du mur. La laine sent un peu la pluie. Ton manteau va là, dans le rang. Les bottes font une petite file. Les miennes sont rouges. Oui, les rouges, près de la porte. Tu tiens ma manche, Sarah ? Oui, papa. Un banc de bois attend sous les manteaux. Le bois est froid. C'est le banc de l'entrée. Le tapis de la classe attend, un peu rêche. Des cartes d'animaux y sont posées, faces ouvertes. Des bêtes, maman ! Tu les vois, sur le tapis ? Une carte montre un chat, les oreilles hautes. Le chat, je le vois. À côté, une tortue garde la tête rentrée. Sur la carte, un &lt;emphasis&gt;éclat de carte&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, sur le papier ? Sarah touche l'éclat de carte. Le papier est lisse, un peu froid. Elle est froide, la tortue. Je lui parle, maintenant ! Tu restes près de nous ? Oui, maman. Tu lui parles, à la tortue ? Oui, très fort ! En ce moment, Sarah se penche sur les cartes. Tortue, tu marches ! Sa voix part trop fort, trop vite. Les cartes glissent sur le tapis. Oh. La tortue disparaît sous une autre carte. L'éclat n'est plus là. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Je la prends ! La carte est sous les autres. Tu la vois, Sarah ? Les épaules de Sarah tombent un peu. Ça serre, dans son ventre. Papa se baisse à sa hauteur. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>répéter</t>
+          <t>éclat de carte</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,39 +1326,61 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_parler_aux_cartes_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Un soleil de doigt dort sur la vitre.
-narrateur|Il a trois rayons, un peu flous.
-narrateur|Le tapis sent encore le savon.
-narrateur|Une carte dépasse d'un sac.
-narrateur|C'est une oreille de chat, toute grise.
-papa|Tu as vu le soleil, Sarah ?
-enfant-f|Il est sur la vitre.
-enfant-f|Il a trois rayons.
-papa|Oui.
-papa|Un petit soleil de doigt.
-narrateur|En ce moment, papa ouvre la porte.
-narrateur|Sarah entre avec lui.
-narrateur|Les chaussures font un bruit doux.
-enfant-f|Je veux la tortue.
-enfant-f|Elle va jusqu'au soleil.
-papa|Tu la fais marcher, alors.
-narrateur|Des cartes d'animaux attendent sur le tapis.
-narrateur|Un sac est ouvert, tout bas.
-narrateur|Raphaël reste près du mur.
-narrateur|Ses mains touchent le crépi, tout doux.
-narrateur|Il ne vient pas encore.
-enfant-f|Raphaël.
-enfant-f|Tu viens ?
-narrateur|Raphaël ne bouge pas.
-narrateur|Il regarde le sac, sans avancer.
-papa|Il a besoin de calme.
-papa|Tu peux dire comment on joue.
-narrateur|Sarah s'arrête au bord du tapis.
-narrateur|La carte du chat dépasse encore.
-narrateur|Le soleil de doigt attend sur la vitre.</t>
+          <t>narrateur|La vitre de la classe est floue.
+narrateur|Un doigt y a tracé un soleil rond.
+enfant-f|Il a trois rayons, papa.
+papa|Tu le vois, Sarah ?
+narrateur|Les manteaux pendent en rang, près du mur.
+narrateur|La laine sent un peu la pluie.
+maman|Ton manteau va là, dans le rang.
+narrateur|Les bottes font une petite file.
+enfant-f|Les miennes sont rouges.
+maman|Oui, les rouges, près de la porte.
+papa|Tu tiens ma manche, Sarah ?
+enfant-f|Oui, papa.
+narrateur|Un banc de bois attend sous les manteaux.
+enfant-f|Le bois est froid.
+papa|C'est le banc de l'entrée.
+narrateur|Le tapis de la classe attend, un peu rêche.
+narrateur|Des cartes d'animaux y sont posées, faces ouvertes.
+enfant-f|Des bêtes, maman !
+maman|Tu les vois, sur le tapis ?
+narrateur|Une carte montre un chat, les oreilles hautes.
+enfant-f|Le chat, je le vois.
+narrateur|À côté, une tortue garde la tête rentrée.
+narrateur|Sur la carte, un éclat de carte brille.
+enfant-f|Il brille, papa.
+papa|Tu le vois, sur le papier ?
+narrateur|Sarah touche l'éclat de carte.
+narrateur|Le papier est lisse, un peu froid.
+enfant-f|Elle est froide, la tortue.
+enfant-f|Je lui parle, maintenant !
+maman|Tu restes près de nous ?
+enfant-f|Oui, maman.
+papa|Tu lui parles, à la tortue ?
+enfant-f|Oui, très fort !
+narrateur|En ce moment, Sarah se penche sur les cartes.
+enfant-f|Tortue, tu marches !
+narrateur|Sa voix part trop fort, trop vite.
+narrateur|Les cartes glissent sur le tapis.
+enfant-f|Oh.
+narrateur|La tortue disparaît sous une autre carte.
+narrateur|L'éclat n'est plus là.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+enfant-f|Je la prends !
+maman|La carte est sous les autres.
+papa|Tu la vois, Sarah ?
+narrateur|Les épaules de Sarah tombent un peu.
+narrateur|Ça serre, dans son ventre.
+narrateur|Papa se baisse à sa hauteur.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1390,17 +1412,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a besoin de calme. Que peut-on faire ?</t>
+          <t>Sarah a besoin de calme. Que peut-on faire ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Raphaël a besoin de calme. Que peut-on faire ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah a besoin de &lt;emphasis level="moderate"&gt;calme&lt;/emphasis&gt;. Que peut-on faire ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Iris a besoin de calme. Que peut-on faire ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Sarah a besoin de &lt;emphasis&gt;calme&lt;/emphasis&gt;. Que peut-on faire ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1425,7 +1447,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>On peut répéter. On peut observer d'abord. Que fait-on ?</t>
+          <t>On peut répéter. Que peut-on faire ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1463,7 +1485,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1474,7 +1496,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1489,34 +1511,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>calme</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1531,22 +1557,22 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=on_dit_le_mot_une_seconde_fois; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Raphaël a besoin de calme.
+          <t>narrateur|Sarah a besoin de calme.
 narrateur|Que peut-on faire ?</t>
         </is>
       </c>
@@ -1574,17 +1600,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah va près du mur. Elle parle tout doux. On pioche une carte. On fait marcher l'animal. Puis on repose. Tu as su répéter. Raphaël écoute. Il va observer d'abord. Il reste près du mur. Sarah retourne au tapis. Elle pioche le chat. Elle marche sur la pointe, tout lentement. Raphaël suit des yeux. Il ne joue pas encore. Observer d'abord, c'est possible. Plus tard, Raphaël tend la main. Il pioche une carte. C'est la tortue. Elle va au soleil. Raphaël avance très lentement. Sarah laisse l'espace. La tortue arrive sous la vitre. Le soleil de doigt a un peu bougé. Bravo, Sarah. Tu as laissé le temps. La tortue est arrivée.</t>
+          <t>Sarah avance trop vite vers le tapis. Tortue, maintenant ! Sa voix se mélange au bruit des bottes. Oh. Les cartes restent en tas. Elle refuse de foncer. Sarah referme la main. Elle regarde le tapis, un instant. Tu veux venir près de la carte ? Papa s'accroupit à la même hauteur. Sarah pose un genou près du tapis. Le tapis est rêche, un peu froid. Tortue. Elle dit le mot plus bas. Tortue. Papa dit le mot, comme elle. Tortue. Sarah dit le mot, une seconde fois. Merci, Sarah. Maman a entendu toute la phrase. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, papa. Sarah écarte les cartes, sans les jeter. La tortue revient, sur le papier. Elle est là. Elle t'écoute. Sarah pose un doigt près de la tortue. Le papier est un peu froid.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah va près du mur. Elle parle tout doux. On pioche une carte. On fait marcher l'animal. Puis on repose. Tu as su répéter. Raphaël écoute. Il va observer d'abord. Il reste près du mur. Sarah retourne au tapis. Elle pioche le chat. Elle marche sur la pointe, tout lentement. Raphaël suit des yeux. Il ne joue pas encore. Observer d'abord, c'est possible. Plus tard, Raphaël tend la main. Il pioche une carte. C'est la tortue. Elle va au soleil. Raphaël avance très lentement. Sarah laisse l'espace. La tortue arrive sous la vitre. Le soleil de doigt a un peu bougé. Bravo, Sarah. Tu as laissé le temps. La tortue est arrivée.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah avance trop vite vers le tapis. &lt;emphasis level="moderate"&gt;Tortue&lt;/emphasis&gt;, maintenant ! Sa voix se mélange au bruit des bottes. Oh. Les cartes restent en tas. Elle refuse de foncer. Sarah referme la main. Elle regarde le tapis, un instant. Tu veux venir près de la carte ? Papa s'accroupit à la même hauteur. Sarah pose un genou près du tapis. Le tapis est rêche, un peu froid. Tortue. Elle dit le mot plus bas. Tortue. Papa dit le mot, comme elle. Tortue. Sarah dit le mot, une seconde fois. Merci, Sarah. Maman a entendu toute la phrase. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, papa. Sarah écarte les cartes, sans les jeter. La tortue revient, sur le papier. Elle est là. Elle t'écoute. Sarah pose un doigt près de la tortue. Le papier est un peu froid.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Zoé a su &lt;emphasis&gt;répéter&lt;/emphasis&gt;. Iris a pu observer d'abord. Le jeu a continué, sans forcer. [pause]</t>
+          <t>Sarah avance trop vite vers le tapis. &lt;emphasis&gt;Tortue&lt;/emphasis&gt;, maintenant ! Sa voix se mélange au bruit des bottes. Oh. Les cartes restent en tas. Elle refuse de foncer. Sarah referme la main. Elle regarde le tapis, un instant. Tu veux venir près de la carte ? Papa s'accroupit à la même hauteur. Sarah pose un genou près du tapis. Le tapis est rêche, un peu froid. Tortue. Elle dit le mot plus bas. Tortue. Papa dit le mot, comme elle. Tortue. Sarah dit le mot, une seconde fois. Merci, Sarah. Maman a entendu toute la phrase. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. Tu as les mains au chaud ? Un peu, papa. Sarah écarte les cartes, sans les jeter. La tortue revient, sur le papier. Elle est là. Elle t'écoute. Sarah pose un doigt près de la tortue. Le papier est un peu froid. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1642,7 +1668,7 @@
         <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1665,7 +1691,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>répéter</t>
+          <t>Tortue</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1679,16 +1705,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1713,42 +1739,46 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=soulagement_prudent; intensite=1; destinataire=enfant; sous_texte=la_voix_forte_echoue_le_mot_revient_plus_bas; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah va près du mur.
-narrateur|Elle parle tout doux.
-enfant-f|On pioche une carte.
-enfant-f|On fait marcher l'animal.
-enfant-f|Puis on repose.
-papa|Tu as su répéter.
-narrateur|Raphaël écoute.
-narrateur|Il va observer d'abord.
-narrateur|Il reste près du mur.
-narrateur|Sarah retourne au tapis.
-narrateur|Elle pioche le chat.
-narrateur|Elle marche sur la pointe, tout lentement.
-narrateur|Raphaël suit des yeux.
-narrateur|Il ne joue pas encore.
-papa|Observer d'abord, c'est possible.
-narrateur|Plus tard, Raphaël tend la main.
-narrateur|Il pioche une carte.
-narrateur|C'est la tortue.
-enfant-f|Elle va au soleil.
-narrateur|Raphaël avance très lentement.
-narrateur|Sarah laisse l'espace.
-narrateur|La tortue arrive sous la vitre.
-narrateur|Le soleil de doigt a un peu bougé.
-papa|Bravo, Sarah.
-papa|Tu as laissé le temps.
-enfant-f|La tortue est arrivée.</t>
+          <t>narrateur|Sarah avance trop vite vers le tapis.
+enfant-f|Tortue, maintenant !
+narrateur|Sa voix se mélange au bruit des bottes.
+enfant-f|Oh.
+narrateur|Les cartes restent en tas.
+narrateur|Elle refuse de foncer.
+narrateur|Sarah referme la main.
+narrateur|Elle regarde le tapis, un instant.
+papa|Tu veux venir près de la carte ?
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Sarah pose un genou près du tapis.
+narrateur|Le tapis est rêche, un peu froid.
+enfant-f|Tortue.
+narrateur|Elle dit le mot plus bas.
+papa|Tortue.
+narrateur|Papa dit le mot, comme elle.
+enfant-f|Tortue.
+narrateur|Sarah dit le mot, une seconde fois.
+maman|Merci, Sarah.
+narrateur|Maman a entendu toute la phrase.
+narrateur|Le ventre de Sarah se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|Tu as les mains au chaud ?
+enfant-f|Un peu, papa.
+narrateur|Sarah écarte les cartes, sans les jeter.
+narrateur|La tortue revient, sur le papier.
+enfant-f|Elle est là.
+maman|Elle t'écoute.
+narrateur|Sarah pose un doigt près de la tortue.
+narrateur|Le papier est un peu froid.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>cartes</t>
+          <t>tapis,cartes</t>
         </is>
       </c>
     </row>
@@ -1775,17 +1805,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sarah range le sac. Raphaël range la tortue, tout doux. Tu as fini de ranger, Sarah ? Oui, papa. Raphaël fait un petit signe. À demain. Les chaussures attendent près de la porte. Le soir, la maison sent la soupe. Tu as joué aux cartes ? La tortue a marché. Jusqu'au soleil. Raphaël était avec toi ? Il a regardé d'abord. Sarah a répété la règle. C'est pour ça, alors. Le soleil de doigt n'est plus à la maison. Il est resté sur la vitre de la classe. La tortue l'a rejoint. Oui. Tout doucement.</t>
+          <t>Sarah tire la carte trop vite. Tu marches jusqu'au soleil ! La carte glisse sous le manteau du rang. Oh. Sarah avance la main. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Sarah observe le tapis, écoute la classe. Sur le papier, un éclat de carte luit. Là, près du soleil de doigt. Sarah tient la carte des deux mains. Le papier est lisse, un peu froid. Elle est froide, papa. Tu la portes jusqu'à la vitre ? Oui, papa. On avance ? Oui, maman. Sarah pose la tortue sous le soleil de doigt. Le papier touche le bois froid de la table. L'air froid revient sur les joues. Sarah serre la carte contre elle. Elle reste froide. On marche. La carte penche, puis se cale. Je la tiens. On avance. Sarah passe le long des manteaux. La laine gratte, un peu.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sarah range le sac. Raphaël range la tortue, tout doux. Tu as fini de ranger, Sarah ? Oui, papa. Raphaël fait un petit signe. À demain. Les chaussures attendent près de la porte. Le soir, la maison sent la soupe. Tu as joué aux cartes ? La tortue a marché. Jusqu'au soleil. Raphaël était avec toi ? Il a regardé d'abord. Sarah a répété la règle. C'est pour ça, alors. Le soleil de doigt n'est plus à la maison. Il est resté sur la vitre de la classe. La tortue l'a rejoint. Oui. Tout doucement.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah tire la carte trop vite. Tu marches jusqu'au soleil ! La carte glisse sous le manteau du rang. Oh. Sarah avance la main. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Sarah observe le tapis, écoute la classe. Sur le papier, un &lt;emphasis level="moderate"&gt;éclat de carte&lt;/emphasis&gt; luit. Là, près du soleil de doigt. Sarah tient la carte des deux mains. Le papier est lisse, un peu froid. Elle est froide, papa. Tu la portes jusqu'à la vitre ? Oui, papa. On avance ? Oui, maman. Sarah pose la tortue sous le soleil de doigt. Le papier touche le bois froid de la table. L'air froid revient sur les joues. Sarah serre la carte contre elle. Elle reste froide. On marche. La carte penche, puis se cale. Je la tiens. On avance. Sarah passe le long des manteaux. La laine gratte, un peu.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Papa reprend Zoé à la porte. Iris range une carte. Elle fait un petit signe. Zoé dit : à de&lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Sarah tire la carte trop vite. Tu marches jusqu'au soleil ! La carte glisse sous le manteau du rang. Oh. Sarah avance la main. Puis elle s'arrête net. Attends, je regarde. Papa attend, sans parler. Sarah observe le tapis, écoute la classe. Sur le papier, un &lt;emphasis&gt;éclat de carte&lt;/emphasis&gt; luit. Là, près du soleil de doigt. Sarah tient la carte des deux mains. Le papier est lisse, un peu froid. Elle est froide, papa. Tu la portes jusqu'à la vitre ? Oui, papa. On avance ? Oui, maman. Sarah pose la tortue sous le soleil de doigt. Le papier touche le bois froid de la table. L'air froid revient sur les joues. Sarah serre la carte contre elle. Elle reste froide. On marche. La carte penche, puis se cale. Je la tiens. On avance. Sarah passe le long des manteaux. La laine gratte, un peu. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1832,7 +1862,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1840,10 +1870,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1866,30 +1896,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de carte</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1898,10 +1928,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1912,34 +1942,47 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_sans_regarder_l_eclat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Sarah range le sac.
-narrateur|Raphaël range la tortue, tout doux.
-papa|Tu as fini de ranger, Sarah ?
+          <t>narrateur|Sarah tire la carte trop vite.
+enfant-f|Tu marches jusqu'au soleil !
+narrateur|La carte glisse sous le manteau du rang.
+enfant-f|Oh.
+narrateur|Sarah avance la main.
+narrateur|Puis elle s'arrête net.
+enfant-f|Attends, je regarde.
+narrateur|Papa attend, sans parler.
+narrateur|Sarah observe le tapis, écoute la classe.
+narrateur|Sur le papier, un éclat de carte luit.
+enfant-f|Là, près du soleil de doigt.
+narrateur|Sarah tient la carte des deux mains.
+narrateur|Le papier est lisse, un peu froid.
+enfant-f|Elle est froide, papa.
+papa|Tu la portes jusqu'à la vitre ?
 enfant-f|Oui, papa.
-narrateur|Raphaël fait un petit signe.
-enfant-f|À demain.
-narrateur|Les chaussures attendent près de la porte.
-narrateur|Le soir, la maison sent la soupe.
-maman|Tu as joué aux cartes ?
-enfant-f|La tortue a marché.
-enfant-f|Jusqu'au soleil.
-maman|Raphaël était avec toi ?
-enfant-f|Il a regardé d'abord.
-papa|Sarah a répété la règle.
-maman|C'est pour ça, alors.
-narrateur|Le soleil de doigt n'est plus à la maison.
-narrateur|Il est resté sur la vitre de la classe.
-enfant-f|La tortue l'a rejoint.
-maman|Oui.
-maman|Tout doucement.</t>
+maman|On avance ?
+enfant-f|Oui, maman.
+narrateur|Sarah pose la tortue sous le soleil de doigt.
+narrateur|Le papier touche le bois froid de la table.
+narrateur|L'air froid revient sur les joues.
+narrateur|Sarah serre la carte contre elle.
+enfant-f|Elle reste froide.
+papa|On marche.
+narrateur|La carte penche, puis se cale.
+enfant-f|Je la tiens.
+maman|On avance.
+narrateur|Sarah passe le long des manteaux.
+narrateur|La laine gratte, un peu.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>porte,soupe</t>
+          <t>porte_classe,tapis</t>
         </is>
       </c>
     </row>
@@ -1966,17 +2009,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La soupe fume encore un peu. La tortue est restée à l'école. Bonne soirée, Sarah. Le soleil avait trois rayons.</t>
+          <t>Le soleil brillait, papa. Tu le vois, comme sur la vitre ? Oui, un peu flou. Sarah pose la carte contre le manteau. On la garde près de nous ? Oui, maman. La classe sentait la laine. Elle est derrière nous. Un soleil de doigt n'est plus aussi net. Sarah respire, plus large. On rentre ? Oui. Les joues de Sarah se réchauffent. La carte reste froide sous la main. Un éclat de carte reste pâle.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La soupe fume encore un peu. La tortue est restée à l'école. Bonne soirée, Sarah. Le soleil avait trois rayons.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le soleil brillait, papa. Tu le vois, comme sur la vitre ? Oui, un peu flou. Sarah pose la carte contre le manteau. On la garde près de nous ? Oui, maman. La classe sentait la laine. Elle est derrière nous. Un soleil de doigt n'est plus aussi net. Sarah respire, plus large. On rentre ? Oui. Les joues de Sarah se réchauffent. La carte reste froide sous la main. Un &lt;emphasis level="moderate"&gt;éclat de carte&lt;/emphasis&gt; reste pâle.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le soleil brillait, papa. Tu le vois, comme sur la vitre ? Oui, un peu flou. Sarah pose la carte contre le manteau. On la garde près de nous ? Oui, maman. La classe sentait la laine. Elle est derrière nous. Un soleil de doigt n'est plus aussi net. Sarah respire, plus large. On rentre ? Oui. Les joues de Sarah se réchauffent. La carte reste froide sous la main. Un &lt;emphasis&gt;éclat de carte&lt;/emphasis&gt; reste pâle.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2023,7 +2066,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2031,10 +2074,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2043,12 +2086,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2057,17 +2100,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de carte</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2076,11 +2123,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2089,27 +2136,47 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pale; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|La soupe fume encore un peu.
-narrateur|La tortue est restée à l'école.
-maman|Bonne soirée, Sarah.
-papa|Le soleil avait trois rayons.</t>
+          <t>enfant-f|Le soleil brillait, papa.
+papa|Tu le vois, comme sur la vitre ?
+enfant-f|Oui, un peu flou.
+narrateur|Sarah pose la carte contre le manteau.
+maman|On la garde près de nous ?
+enfant-f|Oui, maman.
+enfant-f|La classe sentait la laine.
+maman|Elle est derrière nous.
+narrateur|Un soleil de doigt n'est plus aussi net.
+narrateur|Sarah respire, plus large.
+papa|On rentre ?
+enfant-f|Oui.
+narrateur|Les joues de Sarah se réchauffent.
+narrateur|La carte reste froide sous la main.
+narrateur|Un éclat de carte reste pâle.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>porte_classe</t>
         </is>
       </c>
     </row>
@@ -2130,7 +2197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2187,6 +2254,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>